<commit_message>
Örnek veride 'gerçek değildir' notları kaldırıldı, yalnız 'Örnek'; ekran görüntüleri yenilendi; lab eşitleme
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab/ornek/fx-blotter-ornek-sonuc.xlsx
+++ b/lab/ornek/fx-blotter-ornek-sonuc.xlsx
@@ -89,7 +89,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENTETİK ÖRNEK. Gerçek veri değildir, yatırım önerisi değildir. Kalibre Markets tarafından üretildi.</t>
+          <t xml:space="preserve">Örnek.</t>
         </is>
       </c>
     </row>
@@ -299,7 +299,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kullanılan girdiler (sentetik)</t>
+          <t xml:space="preserve">Kullanılan girdiler</t>
         </is>
       </c>
     </row>

</xml_diff>